<commit_message>
Added algorithm to determine symmetry operations
1) Finds determinant
2) Uses Trace(M) and sum of non-diagonals to fish out identity and inversion
3) Looks at diagonals to find axis of rotation or plane normal. This causes issues for cases without diagonals (e.g. 010 001 100)
4) Checks translation part to find space or point
(with other operations within)
</commit_message>
<xml_diff>
--- a/Timeliste - August.xlsx
+++ b/Timeliste - August.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09CA697F-64CA-458F-8310-C19A03ED77C8}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33955753-7337-4C1F-9787-55236DF79605}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>NAVN</t>
   </si>
@@ -87,9 +87,6 @@
   </si>
   <si>
     <t>Timeliste for Sommerjobb 2021</t>
-  </si>
-  <si>
-    <t>start 10 min earlier</t>
   </si>
   <si>
     <t>August</t>
@@ -886,7 +883,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="34" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C6" s="34"/>
       <c r="D6" s="34"/>
@@ -952,32 +949,40 @@
       </c>
     </row>
     <row r="12" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
-      <c r="B12" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="7" t="str">
+      <c r="A12" s="5">
+        <v>44410</v>
+      </c>
+      <c r="B12" s="6">
+        <v>0.48958333333333331</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.65625</v>
+      </c>
+      <c r="D12" s="7">
         <f t="shared" ref="D12:D29" si="0">IF(OR(ISBLANK($B12),ISBLANK($C12))," ",$C12-$B12)</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E12" s="8" t="str">
+        <v>0.16666666666666669</v>
+      </c>
+      <c r="E12" s="8">
         <f t="shared" ref="E12:E29" si="1">IF(OR(ISBLANK($B12),ISBLANK($C12))," ",($C12-$B12)*24)</f>
-        <v xml:space="preserve"> </v>
+        <v>4</v>
       </c>
       <c r="F12" s="9"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E13" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="B13" s="6">
+        <v>0.6875</v>
+      </c>
+      <c r="C13" s="6">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D13" s="7">
+        <f t="shared" si="0"/>
+        <v>0.10416666666666663</v>
+      </c>
+      <c r="E13" s="8">
+        <f t="shared" si="1"/>
+        <v>2.4999999999999991</v>
       </c>
       <c r="F13" s="9"/>
     </row>
@@ -1268,7 +1273,7 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>0</v>
+        <v>0.27083333333333331</v>
       </c>
       <c r="E34" s="38"/>
       <c r="F34" s="39"/>
@@ -1282,13 +1287,13 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>0</v>
+        <v>6.4999999999999991</v>
       </c>
       <c r="E35" s="40"/>
       <c r="F35" s="41"/>
       <c r="H35" s="28">
         <f>55-D35</f>
-        <v>55</v>
+        <v>48.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Evaluating of symmetry and creation of unit cell progress
Mostly fixed EvalSymmetry(), developed CreateCrystal() but need to get corners/edges/faces from old CreateCell(), and tag atoms with symmetry for highlighting appropriately
</commit_message>
<xml_diff>
--- a/Timeliste - August.xlsx
+++ b/Timeliste - August.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33955753-7337-4C1F-9787-55236DF79605}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CC3D800-E91C-48FF-87F3-BBA7D58F9531}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -969,76 +969,102 @@
       <c r="F12" s="9"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A13" s="5"/>
+      <c r="A13" s="5">
+        <v>44410</v>
+      </c>
       <c r="B13" s="6">
         <v>0.6875</v>
       </c>
       <c r="C13" s="6">
-        <v>0.79166666666666663</v>
+        <v>0.79513888888888884</v>
       </c>
       <c r="D13" s="7">
         <f t="shared" si="0"/>
-        <v>0.10416666666666663</v>
+        <v>0.10763888888888884</v>
       </c>
       <c r="E13" s="8">
         <f t="shared" si="1"/>
-        <v>2.4999999999999991</v>
+        <v>2.5833333333333321</v>
       </c>
       <c r="F13" s="9"/>
     </row>
     <row r="14" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A14" s="5"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E14" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A14" s="5">
+        <v>44411</v>
+      </c>
+      <c r="B14" s="6">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0.59027777777777779</v>
+      </c>
+      <c r="D14" s="7">
+        <f t="shared" si="0"/>
+        <v>0.13194444444444448</v>
+      </c>
+      <c r="E14" s="8">
+        <f t="shared" si="1"/>
+        <v>3.1666666666666674</v>
       </c>
       <c r="F14" s="9"/>
     </row>
     <row r="15" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A15" s="5"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E15" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A15" s="5">
+        <v>44411</v>
+      </c>
+      <c r="B15" s="6">
+        <v>0.65625</v>
+      </c>
+      <c r="C15" s="6">
+        <v>0.71875</v>
+      </c>
+      <c r="D15" s="7">
+        <f t="shared" si="0"/>
+        <v>6.25E-2</v>
+      </c>
+      <c r="E15" s="8">
+        <f t="shared" si="1"/>
+        <v>1.5</v>
       </c>
       <c r="F15" s="9"/>
     </row>
     <row r="16" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A16" s="5"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E16" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A16" s="5">
+        <v>44412</v>
+      </c>
+      <c r="B16" s="6">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="C16" s="6">
+        <v>0.67361111111111116</v>
+      </c>
+      <c r="D16" s="7">
+        <f t="shared" si="0"/>
+        <v>0.19444444444444448</v>
+      </c>
+      <c r="E16" s="8">
+        <f t="shared" si="1"/>
+        <v>4.6666666666666679</v>
       </c>
       <c r="F16" s="9"/>
     </row>
     <row r="17" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A17" s="5"/>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E17" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A17" s="5">
+        <v>44413</v>
+      </c>
+      <c r="B17" s="6">
+        <v>0.4548611111111111</v>
+      </c>
+      <c r="C17" s="6">
+        <v>0.57986111111111105</v>
+      </c>
+      <c r="D17" s="7">
+        <f t="shared" si="0"/>
+        <v>0.12499999999999994</v>
+      </c>
+      <c r="E17" s="8">
+        <f t="shared" si="1"/>
+        <v>2.9999999999999987</v>
       </c>
       <c r="F17" s="9"/>
     </row>
@@ -1273,7 +1299,7 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>0.27083333333333331</v>
+        <v>0.78819444444444442</v>
       </c>
       <c r="E34" s="38"/>
       <c r="F34" s="39"/>
@@ -1287,13 +1313,13 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>6.4999999999999991</v>
+        <v>18.916666666666668</v>
       </c>
       <c r="E35" s="40"/>
       <c r="F35" s="41"/>
       <c r="H35" s="28">
         <f>55-D35</f>
-        <v>48.5</v>
+        <v>36.083333333333329</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EvalSymmetry done, CreateCell near end
Even better fixes to EvalSymmetry, did most of CreateCrystal incl. tagging atoms with symmetries,, but need to create corners etc. in relation to bravais lattice and not cartesian version of lattice. After CreateCell I will visualize symmetries. Hope I don't need to re-make with fractional coords., though I see it can simplify as that just means running everything through a bravaisMatrix in the end
</commit_message>
<xml_diff>
--- a/Timeliste - August.xlsx
+++ b/Timeliste - August.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CC3D800-E91C-48FF-87F3-BBA7D58F9531}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E319E8BD-E521-4842-944A-E6CABC9D4E7A}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -419,7 +419,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -471,6 +471,9 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -831,14 +834,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="33"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="34"/>
     </row>
     <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -870,25 +873,25 @@
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="35"/>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="36"/>
     </row>
     <row r="6" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="34"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="35"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="36"/>
     </row>
     <row r="7" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
@@ -1069,30 +1072,42 @@
       <c r="F17" s="9"/>
     </row>
     <row r="18" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A18" s="5"/>
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E18" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A18" s="5">
+        <v>44414</v>
+      </c>
+      <c r="B18" s="6">
+        <v>0.52777777777777779</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0.65625</v>
+      </c>
+      <c r="D18" s="7">
+        <f t="shared" si="0"/>
+        <v>0.12847222222222221</v>
+      </c>
+      <c r="E18" s="8">
+        <f t="shared" si="1"/>
+        <v>3.083333333333333</v>
       </c>
       <c r="F18" s="9"/>
     </row>
     <row r="19" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A19" s="5"/>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E19" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A19" s="5">
+        <v>44414</v>
+      </c>
+      <c r="B19" s="6">
+        <v>0.69444444444444453</v>
+      </c>
+      <c r="C19" s="31">
+        <v>0.86111111111111116</v>
+      </c>
+      <c r="D19" s="7">
+        <f t="shared" si="0"/>
+        <v>0.16666666666666663</v>
+      </c>
+      <c r="E19" s="8">
+        <f t="shared" si="1"/>
+        <v>3.9999999999999991</v>
       </c>
       <c r="F19" s="9"/>
     </row>
@@ -1285,10 +1300,10 @@
       <c r="D33" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="E33" s="36" t="s">
+      <c r="E33" s="37" t="s">
         <v>16</v>
       </c>
-      <c r="F33" s="37"/>
+      <c r="F33" s="38"/>
       <c r="H33" s="30"/>
     </row>
     <row r="34" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
@@ -1299,10 +1314,10 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>0.78819444444444442</v>
-      </c>
-      <c r="E34" s="38"/>
-      <c r="F34" s="39"/>
+        <v>1.0833333333333333</v>
+      </c>
+      <c r="E34" s="39"/>
+      <c r="F34" s="40"/>
       <c r="H34" s="29"/>
     </row>
     <row r="35" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
@@ -1313,13 +1328,13 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>18.916666666666668</v>
-      </c>
-      <c r="E35" s="40"/>
-      <c r="F35" s="41"/>
+        <v>26</v>
+      </c>
+      <c r="E35" s="41"/>
+      <c r="F35" s="42"/>
       <c r="H35" s="28">
         <f>55-D35</f>
-        <v>36.083333333333329</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added gridLines, but encountering issue with corner/edge/face
Changing strategy. Will duplicate cell and translate, then delete those outside 1st cell
</commit_message>
<xml_diff>
--- a/Timeliste - August.xlsx
+++ b/Timeliste - August.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E319E8BD-E521-4842-944A-E6CABC9D4E7A}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19FC1964-6401-47E5-BA3D-621C59DBB431}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -1099,35 +1099,45 @@
         <v>0.69444444444444453</v>
       </c>
       <c r="C19" s="31">
-        <v>0.86111111111111116</v>
+        <v>0.88194444444444453</v>
       </c>
       <c r="D19" s="7">
         <f t="shared" si="0"/>
-        <v>0.16666666666666663</v>
+        <v>0.1875</v>
       </c>
       <c r="E19" s="8">
         <f t="shared" si="1"/>
-        <v>3.9999999999999991</v>
+        <v>4.5</v>
       </c>
       <c r="F19" s="9"/>
     </row>
     <row r="20" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A20" s="5"/>
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E20" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A20" s="5">
+        <v>44417</v>
+      </c>
+      <c r="B20" s="6">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="C20" s="6">
+        <v>0.6875</v>
+      </c>
+      <c r="D20" s="7">
+        <f t="shared" si="0"/>
+        <v>0.14583333333333337</v>
+      </c>
+      <c r="E20" s="8">
+        <f t="shared" si="1"/>
+        <v>3.5000000000000009</v>
       </c>
       <c r="F20" s="9"/>
     </row>
     <row r="21" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
-      <c r="B21" s="6"/>
+      <c r="A21" s="5">
+        <v>44417</v>
+      </c>
+      <c r="B21" s="6">
+        <v>0.70833333333333337</v>
+      </c>
       <c r="C21" s="6"/>
       <c r="D21" s="7" t="str">
         <f t="shared" si="0"/>
@@ -1314,7 +1324,7 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>1.0833333333333333</v>
+        <v>1.25</v>
       </c>
       <c r="E34" s="39"/>
       <c r="F34" s="40"/>
@@ -1328,13 +1338,13 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E35" s="41"/>
       <c r="F35" s="42"/>
       <c r="H35" s="28">
         <f>55-D35</f>
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated symmetry-tagging to use the reciprocal matrix
</commit_message>
<xml_diff>
--- a/Timeliste - August.xlsx
+++ b/Timeliste - August.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19FC1964-6401-47E5-BA3D-621C59DBB431}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44C1A065-8AE4-4511-9D81-5B561ABBCF74}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -1138,20 +1138,26 @@
       <c r="B21" s="6">
         <v>0.70833333333333337</v>
       </c>
-      <c r="C21" s="6"/>
-      <c r="D21" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E21" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="C21" s="6">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="D21" s="7">
+        <f t="shared" si="0"/>
+        <v>0.125</v>
+      </c>
+      <c r="E21" s="8">
+        <f t="shared" si="1"/>
+        <v>3</v>
       </c>
       <c r="F21" s="9"/>
     </row>
     <row r="22" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A22" s="5"/>
-      <c r="B22" s="6"/>
+      <c r="A22" s="5">
+        <v>44418</v>
+      </c>
+      <c r="B22" s="6">
+        <v>0.5</v>
+      </c>
       <c r="C22" s="6"/>
       <c r="D22" s="7" t="str">
         <f t="shared" si="0"/>
@@ -1324,7 +1330,7 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>1.25</v>
+        <v>1.375</v>
       </c>
       <c r="E34" s="39"/>
       <c r="F34" s="40"/>
@@ -1338,13 +1344,13 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E35" s="41"/>
       <c r="F35" s="42"/>
       <c r="H35" s="28">
         <f>55-D35</f>
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implemented visual rotation axes
Drew all rotation-symbols in paint.net and imported them for use as sprites
</commit_message>
<xml_diff>
--- a/Timeliste - August.xlsx
+++ b/Timeliste - August.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44C1A065-8AE4-4511-9D81-5B561ABBCF74}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CF05707-C770-4634-957E-FD423DAEB67F}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -1158,28 +1158,36 @@
       <c r="B22" s="6">
         <v>0.5</v>
       </c>
-      <c r="C22" s="6"/>
-      <c r="D22" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E22" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="C22" s="6">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="D22" s="7">
+        <f t="shared" si="0"/>
+        <v>0.10416666666666663</v>
+      </c>
+      <c r="E22" s="8">
+        <f t="shared" si="1"/>
+        <v>2.4999999999999991</v>
       </c>
       <c r="F22" s="9"/>
     </row>
     <row r="23" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A23" s="5"/>
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E23" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A23" s="5">
+        <v>44418</v>
+      </c>
+      <c r="B23" s="6">
+        <v>0.63194444444444442</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0.73611111111111116</v>
+      </c>
+      <c r="D23" s="7">
+        <f t="shared" si="0"/>
+        <v>0.10416666666666674</v>
+      </c>
+      <c r="E23" s="8">
+        <f t="shared" si="1"/>
+        <v>2.5000000000000018</v>
       </c>
       <c r="F23" s="9"/>
     </row>
@@ -1330,7 +1338,7 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>1.375</v>
+        <v>1.5833333333333333</v>
       </c>
       <c r="E34" s="39"/>
       <c r="F34" s="40"/>
@@ -1344,13 +1352,13 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E35" s="41"/>
       <c r="F35" s="42"/>
       <c r="H35" s="28">
         <f>55-D35</f>
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Push before upgrading Unity
From 2020.3.11f1 to 2020.3.16f1
</commit_message>
<xml_diff>
--- a/Timeliste - August.xlsx
+++ b/Timeliste - August.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23930154-CF79-4D51-B54E-902CC5B1FBA9}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26B5D8CE-8749-4EC6-8FE6-E8DE8A4672F2}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -1252,8 +1252,12 @@
       <c r="F26" s="9"/>
     </row>
     <row r="27" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A27" s="5"/>
-      <c r="B27" s="6"/>
+      <c r="A27" s="5">
+        <v>44431</v>
+      </c>
+      <c r="B27" s="6">
+        <v>0.52083333333333337</v>
+      </c>
       <c r="C27" s="6"/>
       <c r="D27" s="7" t="str">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
Tried adding scaling to player
Did not work, but not too far off
</commit_message>
<xml_diff>
--- a/Timeliste - August.xlsx
+++ b/Timeliste - August.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26B5D8CE-8749-4EC6-8FE6-E8DE8A4672F2}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75D5F820-4CF2-4276-BB9B-EEF1DA071D99}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -1258,14 +1258,16 @@
       <c r="B27" s="6">
         <v>0.52083333333333337</v>
       </c>
-      <c r="C27" s="6"/>
-      <c r="D27" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E27" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="C27" s="6">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="D27" s="7">
+        <f t="shared" si="0"/>
+        <v>0.20833333333333326</v>
+      </c>
+      <c r="E27" s="8">
+        <f t="shared" si="1"/>
+        <v>4.9999999999999982</v>
       </c>
       <c r="F27" s="9"/>
     </row>
@@ -1360,7 +1362,7 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>1.875</v>
+        <v>2.083333333333333</v>
       </c>
       <c r="E34" s="39"/>
       <c r="F34" s="40"/>
@@ -1374,13 +1376,13 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="E35" s="41"/>
       <c r="F35" s="42"/>
       <c r="H35" s="28">
         <f>55-D35</f>
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added growing and shrinking of player
Left Thumbstick: Grow 10%
Right Thumbstick: Shrink 10%
</commit_message>
<xml_diff>
--- a/Timeliste - August.xlsx
+++ b/Timeliste - August.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75D5F820-4CF2-4276-BB9B-EEF1DA071D99}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9950CAC5-F94D-4A83-BA92-6EA19EC83D6D}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -1272,8 +1272,12 @@
       <c r="F27" s="9"/>
     </row>
     <row r="28" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A28" s="5"/>
-      <c r="B28" s="6"/>
+      <c r="A28" s="5">
+        <v>44432</v>
+      </c>
+      <c r="B28" s="6">
+        <v>0.44791666666666669</v>
+      </c>
       <c r="C28" s="6"/>
       <c r="D28" s="7" t="str">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
Added a Runtime File Browser
and began figuring out how it works
</commit_message>
<xml_diff>
--- a/Timeliste - August.xlsx
+++ b/Timeliste - August.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68E35679-6603-4A17-A1D5-6F7419B83243}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9D48CCD-4928-45B9-9680-F646FAD6E07A}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -1292,16 +1292,22 @@
       <c r="F28" s="9"/>
     </row>
     <row r="29" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A29" s="5"/>
-      <c r="B29" s="6"/>
-      <c r="C29" s="6"/>
-      <c r="D29" s="7" t="str">
-        <f t="shared" si="0"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E29" s="8" t="str">
-        <f t="shared" si="1"/>
-        <v xml:space="preserve"> </v>
+      <c r="A29" s="5">
+        <v>44432</v>
+      </c>
+      <c r="B29" s="6">
+        <v>0.6875</v>
+      </c>
+      <c r="C29" s="6">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="D29" s="7">
+        <f t="shared" si="0"/>
+        <v>2.083333333333337E-2</v>
+      </c>
+      <c r="E29" s="8">
+        <f t="shared" si="1"/>
+        <v>0.50000000000000089</v>
       </c>
       <c r="F29" s="9"/>
     </row>
@@ -1368,7 +1374,7 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>2.1979166666666665</v>
+        <v>2.21875</v>
       </c>
       <c r="E34" s="39"/>
       <c r="F34" s="40"/>
@@ -1382,13 +1388,13 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>52.75</v>
+        <v>53.25</v>
       </c>
       <c r="E35" s="41"/>
       <c r="F35" s="42"/>
       <c r="H35" s="28">
         <f>55-D35</f>
-        <v>2.25</v>
+        <v>1.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New FileBrowser works. Will build game this evening
120/120 hours used
</commit_message>
<xml_diff>
--- a/Timeliste - August.xlsx
+++ b/Timeliste - August.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9D48CCD-4928-45B9-9680-F646FAD6E07A}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C5EED1A-183D-4D13-A2C5-5E7FADFEC771}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -1312,16 +1312,22 @@
       <c r="F29" s="9"/>
     </row>
     <row r="30" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A30" s="10"/>
-      <c r="B30" s="6"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="7" t="str">
+      <c r="A30" s="5">
+        <v>44433</v>
+      </c>
+      <c r="B30" s="6">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="C30" s="6">
+        <v>0.59375</v>
+      </c>
+      <c r="D30" s="7">
         <f t="shared" ref="D30:D32" si="2">IF(OR(ISBLANK($B30),ISBLANK($C30))," ",$C30-$B30)</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E30" s="8" t="str">
+        <v>7.291666666666663E-2</v>
+      </c>
+      <c r="E30" s="8">
         <f t="shared" ref="E30:E32" si="3">IF(OR(ISBLANK($B30),ISBLANK($C30))," ",($C30-$B30)*24)</f>
-        <v xml:space="preserve"> </v>
+        <v>1.7499999999999991</v>
       </c>
       <c r="F30" s="9"/>
     </row>
@@ -1374,7 +1380,7 @@
       </c>
       <c r="D34" s="18">
         <f>SUM(D12:D32)</f>
-        <v>2.21875</v>
+        <v>2.2916666666666665</v>
       </c>
       <c r="E34" s="39"/>
       <c r="F34" s="40"/>
@@ -1388,13 +1394,13 @@
       </c>
       <c r="D35" s="22">
         <f>SUM(E12:E32)</f>
-        <v>53.25</v>
+        <v>55</v>
       </c>
       <c r="E35" s="41"/>
       <c r="F35" s="42"/>
       <c r="H35" s="28">
         <f>55-D35</f>
-        <v>1.75</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New build + atomsize change
Works when SteamVR is the OpenXR Runtime, but scripting backend il2cpp does not support external processes (which we use for cif2cell)

Changed atom size from 2*ionradii in Å to 1*ionradii in Å
</commit_message>
<xml_diff>
--- a/Timeliste - August.xlsx
+++ b/Timeliste - August.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erlen\Documents\Github\Crystallographic-Reality\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C5EED1A-183D-4D13-A2C5-5E7FADFEC771}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{115CE4AA-D1B0-4FEE-B561-764C97ACD4E3}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{36930395-203A-46D0-A2AB-0BDFDA6E0730}"/>
   </bookViews>
@@ -419,7 +419,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -436,9 +436,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
@@ -834,14 +831,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -849,7 +846,7 @@
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="24"/>
+      <c r="F2" s="23"/>
     </row>
     <row r="3" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
@@ -857,71 +854,71 @@
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="24"/>
+      <c r="F3" s="23"/>
     </row>
     <row r="4" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="26"/>
+      <c r="F4" s="25"/>
     </row>
     <row r="5" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="35"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="36"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="35"/>
     </row>
     <row r="6" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="35"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="36"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="35"/>
     </row>
     <row r="7" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="27"/>
+      <c r="B7" s="26"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
-      <c r="F7" s="24"/>
+      <c r="F7" s="23"/>
     </row>
     <row r="8" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="27"/>
+      <c r="B8" s="26"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
-      <c r="F8" s="24"/>
+      <c r="F8" s="23"/>
     </row>
     <row r="9" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="27"/>
+      <c r="B9" s="26"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
-      <c r="F9" s="24"/>
+      <c r="F9" s="23"/>
     </row>
     <row r="10" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
@@ -929,7 +926,7 @@
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
-      <c r="F10" s="25"/>
+      <c r="F10" s="24"/>
     </row>
     <row r="11" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
@@ -1098,7 +1095,7 @@
       <c r="B19" s="6">
         <v>0.69444444444444453</v>
       </c>
-      <c r="C19" s="31">
+      <c r="C19" s="30">
         <v>0.88194444444444453</v>
       </c>
       <c r="D19" s="7">
@@ -1332,75 +1329,87 @@
       <c r="F30" s="9"/>
     </row>
     <row r="31" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A31" s="10"/>
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="7" t="str">
+      <c r="A31" s="5">
+        <v>44433</v>
+      </c>
+      <c r="B31" s="6">
+        <v>0.96527777777777779</v>
+      </c>
+      <c r="C31" s="6">
+        <v>0.98611111111111116</v>
+      </c>
+      <c r="D31" s="7">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E31" s="8" t="str">
+        <v>2.083333333333337E-2</v>
+      </c>
+      <c r="E31" s="8">
         <f t="shared" si="3"/>
-        <v xml:space="preserve"> </v>
+        <v>0.50000000000000089</v>
       </c>
       <c r="F31" s="9"/>
     </row>
     <row r="32" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="10"/>
-      <c r="B32" s="6"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="7" t="str">
+      <c r="A32" s="5">
+        <v>44434</v>
+      </c>
+      <c r="B32" s="6">
+        <v>0</v>
+      </c>
+      <c r="C32" s="6">
+        <v>3.125E-2</v>
+      </c>
+      <c r="D32" s="7">
         <f t="shared" si="2"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="E32" s="11" t="str">
+        <v>3.125E-2</v>
+      </c>
+      <c r="E32" s="10">
         <f t="shared" si="3"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="F32" s="12"/>
+        <v>0.75</v>
+      </c>
+      <c r="F32" s="11"/>
     </row>
     <row r="33" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A33" s="13"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="15"/>
-      <c r="D33" s="16" t="s">
+      <c r="A33" s="12"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="E33" s="37" t="s">
+      <c r="E33" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="F33" s="38"/>
-      <c r="H33" s="30"/>
+      <c r="F33" s="37"/>
+      <c r="H33" s="29"/>
     </row>
     <row r="34" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A34" s="17"/>
-      <c r="B34" s="15"/>
+      <c r="A34" s="16"/>
+      <c r="B34" s="14"/>
       <c r="C34" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D34" s="18">
+      <c r="D34" s="17">
         <f>SUM(D12:D32)</f>
-        <v>2.2916666666666665</v>
-      </c>
-      <c r="E34" s="39"/>
-      <c r="F34" s="40"/>
-      <c r="H34" s="29"/>
+        <v>2.34375</v>
+      </c>
+      <c r="E34" s="38"/>
+      <c r="F34" s="39"/>
+      <c r="H34" s="28"/>
     </row>
     <row r="35" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="19"/>
-      <c r="B35" s="20"/>
-      <c r="C35" s="21" t="s">
+      <c r="A35" s="18"/>
+      <c r="B35" s="19"/>
+      <c r="C35" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="D35" s="22">
+      <c r="D35" s="21">
         <f>SUM(E12:E32)</f>
-        <v>55</v>
-      </c>
-      <c r="E35" s="41"/>
-      <c r="F35" s="42"/>
-      <c r="H35" s="28">
+        <v>56.25</v>
+      </c>
+      <c r="E35" s="40"/>
+      <c r="F35" s="41"/>
+      <c r="H35" s="27">
         <f>55-D35</f>
-        <v>0</v>
+        <v>-1.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>